<commit_message>
Resolve issues with column naming errors
</commit_message>
<xml_diff>
--- a/doc/CEDS DW Version 14.0.0.0 to 14.1.0.0.xlsx
+++ b/doc/CEDS DW Version 14.0.0.0 to 14.1.0.0.xlsx
@@ -483,9 +483,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -518,9 +515,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -553,9 +547,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -588,9 +579,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -623,9 +611,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -658,9 +643,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -693,9 +675,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -708,7 +687,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>JobPositionCancellationReasonCode</t>
+          <t>JobPositionStatusCancelledReasonCode</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -728,9 +707,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -743,7 +719,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>JobPositionCancellationReasonDescription</t>
+          <t>JobPositionStatusCancelledReasonDescription</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -763,9 +739,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -798,9 +771,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -833,9 +803,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -878,7 +845,6 @@
           <t>DimCipCodes</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -921,7 +887,6 @@
           <t>DimCipCodes</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -964,7 +929,6 @@
           <t>DimCipCodes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1007,7 +971,6 @@
           <t>DimCipCodes</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1050,7 +1013,6 @@
           <t>DimCredentialAwards</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1093,7 +1055,6 @@
           <t>DimCredentialDefinitions</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1136,7 +1097,6 @@
           <t>DimCredentialDefinitions</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1179,7 +1139,6 @@
           <t>DimFacilities</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1222,7 +1181,6 @@
           <t>DimFacilityStatuses</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1265,7 +1223,6 @@
           <t>DimFacilityStatuses</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1308,7 +1265,6 @@
           <t>DimFacilityUtilization</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1351,7 +1307,6 @@
           <t>DimFacilityUtilization</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1394,7 +1349,6 @@
           <t>DimK12StaffAssignmentStatuses</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1437,7 +1391,6 @@
           <t>DimK12StaffAssignmentStatuses</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1480,7 +1433,6 @@
           <t>DimProfessionalDevelopmentActivities</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1493,7 +1445,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ProfessionalDevelopmentApprovalStartDate</t>
+          <t>ProfessionalDevelopmentActivityApprovalStartDate</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1523,7 +1475,6 @@
           <t>DimProfessionalDevelopmentActivities</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1536,7 +1487,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>ProfessionalDevelopmentApprovalEndDate</t>
+          <t>ProfessionalDevelopmentActivityApprovalEndDate</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1566,7 +1517,6 @@
           <t>DimSeaJobClassifications</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1609,7 +1559,6 @@
           <t>DimSeaJobClassifications</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1652,7 +1601,6 @@
           <t>FactDirectory</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1695,7 +1643,6 @@
           <t>FactDirectory</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1738,7 +1685,6 @@
           <t>FactK12StaffAssessments</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1781,7 +1727,6 @@
           <t>FactK12StaffAssignments</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1824,7 +1769,6 @@
           <t>FactK12StaffAssignments</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1867,7 +1811,6 @@
           <t>FactK12StaffAssignments</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1910,7 +1853,6 @@
           <t>FactK12StaffAssignments</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1953,7 +1895,6 @@
           <t>FactK12StaffAssignments</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -1996,7 +1937,6 @@
           <t>FactK12StaffCourseSections</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2039,7 +1979,6 @@
           <t>FactK12StaffEmployments</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2082,7 +2021,6 @@
           <t>FactK12StaffEvaluationParts</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2125,7 +2063,6 @@
           <t>FactK12StaffProfessionalDevelopmentSessions</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2168,7 +2105,6 @@
           <t>FactK12StaffProfessionalDevelopmentSessions</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2211,7 +2147,6 @@
           <t>FactK12StaffProfessionalDevelopmentSessions</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2254,7 +2189,6 @@
           <t>FactK12StaffProfessionalDevelopmentSessions</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2297,7 +2231,6 @@
           <t>FactK12StaffProfessionalDevelopmentSessions</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -2340,7 +2273,6 @@
           <t>FactK12StaffProfessionalDevelopmentSessions</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>RDS</t>
@@ -4357,7 +4289,6 @@
           <t>OrganizationAddress</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>Staging</t>

</xml_diff>

<commit_message>
Removed field determined was actually a CEPI extension, not core CEDS.
</commit_message>
<xml_diff>
--- a/doc/CEDS DW Version 14.0.0.0 to 14.1.0.0.xlsx
+++ b/doc/CEDS DW Version 14.0.0.0 to 14.1.0.0.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.66" customWidth="1" min="1" max="1"/>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>NumberOfCreditsEarnedProfessionalDevelopmentDays</t>
+          <t>NumberOfCreditsEarnedProfessionalDevelopmentHours</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>NumberOfCreditsEarnedProfessionalDevelopmentHours</t>
+          <t>NumberOfCreditsEarnedDegreeCredit</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>NumberOfCreditsEarnedDegreeCredit</t>
+          <t>NumberOfCreditsEarnedContinuingEducationUnits</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>NumberOfCreditsEarnedContinuingEducationUnits</t>
+          <t>NumberOfCreditsEarnedClockHours</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2270,7 +2270,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>FactK12StaffProfessionalDevelopmentSessions</t>
+          <t>FactK12StaffAssessments</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>K12StaffPersonId</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2280,12 +2285,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FactK12StaffProfessionalDevelopmentSessions</t>
+          <t>FactK12StaffAssessments</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>NumberOfCreditsEarnedClockHours</t>
+          <t>K12StaffId</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2300,7 +2305,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>New Table and/or Column added</t>
+          <t>Column renamed - standardized staff identifier naming to K12Staff</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2322,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>K12StaffPersonId</t>
+          <t>K12StaffPerson_CurrentId</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2332,7 +2337,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>K12StaffId</t>
+          <t>K12Staff_CurrentId</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2359,12 +2364,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>FactK12StaffAssessments</t>
+          <t>FactK12StaffCourseSections</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>K12StaffPerson_CurrentId</t>
+          <t>K12StaffMemberId</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2374,12 +2379,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FactK12StaffAssessments</t>
+          <t>FactK12StaffCourseSections</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>K12Staff_CurrentId</t>
+          <t>K12StaffId</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2411,7 +2416,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>K12StaffMemberId</t>
+          <t>K12StaffMember_CurrentId</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2426,7 +2431,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>K12StaffId</t>
+          <t>K12Staff_CurrentId</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2453,12 +2458,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>FactK12StaffCourseSections</t>
+          <t>FactK12StaffEmployments</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>K12StaffMember_CurrentId</t>
+          <t>YearsOfPriorTeachingExperience</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2468,12 +2473,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FactK12StaffCourseSections</t>
+          <t>FactK12StaffEmployments</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>K12Staff_CurrentId</t>
+          <t>YearsOfPriorTeachingExperience</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2488,7 +2493,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Column renamed - standardized staff identifier naming to K12Staff</t>
+          <t>Data type widened from decimal(3,2) to decimal(4,2)</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2510,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>YearsOfPriorTeachingExperience</t>
+          <t>YearsOfPriorProfessionalExperience</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2520,7 +2525,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>YearsOfPriorTeachingExperience</t>
+          <t>YearsOfPriorProfessionalExperience</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2552,7 +2557,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>YearsOfPriorProfessionalExperience</t>
+          <t>YearsOfTotalExperience</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2567,7 +2572,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>YearsOfPriorProfessionalExperience</t>
+          <t>YearsOfTotalExperience</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2599,7 +2604,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>YearsOfTotalExperience</t>
+          <t>YearsofPriorAdultEducationTeachingExperience</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2614,7 +2619,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>YearsOfTotalExperience</t>
+          <t>YearsofPriorAdultEducationTeachingExperience</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2646,7 +2651,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>YearsofPriorAdultEducationTeachingExperience</t>
+          <t>ContractDaysOfServicePerYear</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2661,7 +2666,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>YearsofPriorAdultEducationTeachingExperience</t>
+          <t>ContractDaysOfServicePerYear</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2688,12 +2693,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>FactK12StaffEmployments</t>
+          <t>DimCredentialDefinitions</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ContractDaysOfServicePerYear</t>
+          <t>CredentialTypeCode</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2703,12 +2708,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>FactK12StaffEmployments</t>
+          <t>DimCredentialDefinitions</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>ContractDaysOfServicePerYear</t>
+          <t>CredentialTypeCode</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2723,7 +2728,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Data type widened from decimal(3,2) to decimal(4,2)</t>
+          <t>Column nullability changed from NOT NULL to NULL</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2745,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CredentialTypeCode</t>
+          <t>CredentialTypeDescription</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2755,7 +2760,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>CredentialTypeCode</t>
+          <t>CredentialTypeDescription</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2787,7 +2792,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CredentialTypeDescription</t>
+          <t>CredentialDefinitionStatusTypeCode</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2802,7 +2807,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>CredentialTypeDescription</t>
+          <t>CredentialDefinitionStatusTypeCode</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2834,7 +2839,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CredentialDefinitionStatusTypeCode</t>
+          <t>CredentialDefinitionStatusTypeDescription</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2849,7 +2854,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>CredentialDefinitionStatusTypeCode</t>
+          <t>CredentialDefinitionStatusTypeDescription</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2881,7 +2886,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CredentialDefinitionStatusTypeDescription</t>
+          <t>CredentialDefinitionIntendedPurposeTypeCode</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2896,7 +2901,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>CredentialDefinitionStatusTypeDescription</t>
+          <t>CredentialDefinitionIntendedPurposeTypeCode</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2928,7 +2933,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CredentialDefinitionIntendedPurposeTypeCode</t>
+          <t>CredentialDefinitionIntendedPurposeTypeDescription</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2943,7 +2948,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CredentialDefinitionIntendedPurposeTypeCode</t>
+          <t>CredentialDefinitionIntendedPurposeTypeDescription</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2975,7 +2980,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CredentialDefinitionIntendedPurposeTypeDescription</t>
+          <t>CredentialDefinitionAssessmentMethodTypeCode</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2990,7 +2995,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>CredentialDefinitionIntendedPurposeTypeDescription</t>
+          <t>CredentialDefinitionAssessmentMethodTypeCode</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3022,7 +3027,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CredentialDefinitionAssessmentMethodTypeCode</t>
+          <t>CredentialDefinitionAssessmentMethodTypeDescription</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3037,7 +3042,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>CredentialDefinitionAssessmentMethodTypeCode</t>
+          <t>CredentialDefinitionAssessmentMethodTypeDescription</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3069,7 +3074,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CredentialDefinitionAssessmentMethodTypeDescription</t>
+          <t>CTDLAudienceLevelTypeCode</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3084,7 +3089,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>CredentialDefinitionAssessmentMethodTypeDescription</t>
+          <t>CTDLAudienceLevelTypeCode</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3116,7 +3121,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CTDLAudienceLevelTypeCode</t>
+          <t>CTDLAudienceLevelTypeDescription</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3131,7 +3136,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>CTDLAudienceLevelTypeCode</t>
+          <t>CTDLAudienceLevelTypeDescription</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3163,7 +3168,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CTDLAudienceLevelTypeDescription</t>
+          <t>CredentialDefinitionTerminalDegreeIndicatorCode</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3178,7 +3183,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>CTDLAudienceLevelTypeDescription</t>
+          <t>CredentialDefinitionTerminalDegreeIndicatorCode</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3210,7 +3215,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CredentialDefinitionTerminalDegreeIndicatorCode</t>
+          <t>CredentialDefinitionTerminalDegreeIndicatorDescription</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3225,7 +3230,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>CredentialDefinitionTerminalDegreeIndicatorCode</t>
+          <t>CredentialDefinitionTerminalDegreeIndicatorDescription</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3257,7 +3262,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CredentialDefinitionTerminalDegreeIndicatorDescription</t>
+          <t>CredentialDefinitionScedCode</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3272,7 +3277,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>CredentialDefinitionTerminalDegreeIndicatorDescription</t>
+          <t>CredentialDefinitionScedCode</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3304,7 +3309,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CredentialDefinitionScedCode</t>
+          <t>CredentialDefinitionLowGradeLevelCode</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3319,7 +3324,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>CredentialDefinitionScedCode</t>
+          <t>CredentialDefinitionLowGradeLevelCode</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3351,7 +3356,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CredentialDefinitionLowGradeLevelCode</t>
+          <t>CredentialDefinitionHighGradeLevelCode</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3366,7 +3371,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>CredentialDefinitionLowGradeLevelCode</t>
+          <t>CredentialDefinitionHighGradeLevelCode</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3393,12 +3398,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>DimCredentialDefinitions</t>
+          <t>FactDirectory</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CredentialDefinitionHighGradeLevelCode</t>
+          <t>LeaId</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3408,12 +3413,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>DimCredentialDefinitions</t>
+          <t>FactDirectory</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>CredentialDefinitionHighGradeLevelCode</t>
+          <t>LeaId</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3428,7 +3433,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Column nullability changed from NOT NULL to NULL</t>
+          <t>Column changed to NOT NULL with a default of -1</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3450,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>LeaId</t>
+          <t>OrganizationId</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3460,7 +3465,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>LeaId</t>
+          <t>OrganizationId</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3492,7 +3497,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>OrganizationId</t>
+          <t>SeaId</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3507,7 +3512,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>OrganizationId</t>
+          <t>SeaId</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3539,7 +3544,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SeaId</t>
+          <t>PsInstitutionID</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3554,7 +3559,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>SeaId</t>
+          <t>PsInstitutionID</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3586,7 +3591,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>PsInstitutionID</t>
+          <t>IeuId</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3601,7 +3606,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>PsInstitutionID</t>
+          <t>IeuId</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3633,7 +3638,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>IeuId</t>
+          <t>K12SchoolId</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3648,7 +3653,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>IeuId</t>
+          <t>K12SchoolId</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3680,7 +3685,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>K12SchoolId</t>
+          <t>AeProviderId</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3695,7 +3700,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>K12SchoolId</t>
+          <t>AeProviderId</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3727,7 +3732,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AeProviderId</t>
+          <t>ComprehensiveAndTargetedSupportId</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3742,7 +3747,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>AeProviderId</t>
+          <t>ComprehensiveAndTargetedSupportId</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3774,7 +3779,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ComprehensiveAndTargetedSupportId</t>
+          <t>NOrDStatusId</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3789,7 +3794,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>ComprehensiveAndTargetedSupportId</t>
+          <t>NOrDStatusId</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3821,7 +3826,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>NOrDStatusId</t>
+          <t>CharterSchoolManagementOrganizationId</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3836,7 +3841,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>NOrDStatusId</t>
+          <t>CharterSchoolManagementOrganizationId</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3868,7 +3873,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CharterSchoolManagementOrganizationId</t>
+          <t>CharterSchoolStatusId</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3883,7 +3888,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>CharterSchoolManagementOrganizationId</t>
+          <t>CharterSchoolStatusId</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3915,7 +3920,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CharterSchoolStatusId</t>
+          <t>CharterSchoolAuthorizerId</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3930,7 +3935,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>CharterSchoolStatusId</t>
+          <t>CharterSchoolAuthorizerId</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3962,7 +3967,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CharterSchoolAuthorizerId</t>
+          <t>AlternativeSchoolStatusId</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3977,7 +3982,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>CharterSchoolAuthorizerId</t>
+          <t>AlternativeSchoolStatusId</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4009,7 +4014,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AlternativeSchoolStatusId</t>
+          <t>K12SchoolStatusId</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4024,7 +4029,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>AlternativeSchoolStatusId</t>
+          <t>K12SchoolStatusId</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4056,7 +4061,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>K12SchoolStatusId</t>
+          <t>EarlyChildhoodOrganizationStatusId</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4071,7 +4076,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>K12SchoolStatusId</t>
+          <t>EarlyChildhoodOrganizationStatusId</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4103,7 +4108,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>EarlyChildhoodOrganizationStatusId</t>
+          <t>EarlyLearningOrganizationId</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4118,7 +4123,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>EarlyChildhoodOrganizationStatusId</t>
+          <t>EarlyLearningOrganizationId</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4150,7 +4155,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>EarlyLearningOrganizationId</t>
+          <t>DataCollectionId</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4165,7 +4170,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>EarlyLearningOrganizationId</t>
+          <t>DataCollectionId</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4197,7 +4202,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>DataCollectionId</t>
+          <t>SchoolYearId</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4212,7 +4217,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>DataCollectionId</t>
+          <t>SchoolYearId</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4234,32 +4239,27 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RDS</t>
+          <t>Staging</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>FactDirectory</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>SchoolYearId</t>
+          <t>OrganizationAddress</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>RDS</t>
+          <t>Staging</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>FactDirectory</t>
+          <t>OrganizationAddress</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>SchoolYearId</t>
+          <t>AddressCountyName</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4273,48 +4273,6 @@
         </is>
       </c>
       <c r="I89" t="inlineStr">
-        <is>
-          <t>Column changed to NOT NULL with a default of -1</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>Staging</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>OrganizationAddress</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Staging</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>OrganizationAddress</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>AddressCountyName</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>Same</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>Diff</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
         <is>
           <t>New Table and/or Column added</t>
         </is>

</xml_diff>